<commit_message>
Board Outline korrigiert und auf richtiges Layer gezogen, Output Jobs finalisiert
Output Job Files in JLCDFM-Tool überprüft
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_current_measurement_dsub_to_rj45/01/BOM/BOM_JLC-uz_per_current_measurement_dsub_to_rj45.xlsx
+++ b/Project Outputs for uz_per_current_measurement_dsub_to_rj45/01/BOM/BOM_JLC-uz_per_current_measurement_dsub_to_rj45.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_per_current_measurement_dsub_to_rj45_4channel\Project Outputs for uz_per_current_measurement_dsub_to_rj45\01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D14588A2-3873-4534-A251-849254E3B05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E623340-C6C3-416B-A7DD-552F917C7199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{F886B182-FBB2-4DE0-BDEC-3E6D8888F23D}"/>
+    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{9F5170AF-19A8-4807-B0BF-E5ED08A867CC}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_current_measurem" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="120">
   <si>
     <t>Quantity</t>
   </si>
@@ -78,7 +78,7 @@
     <t>1 µF</t>
   </si>
   <si>
-    <t>C1_A, C1_B, C1_C, C1_D, C4, C5, C6, C7, C8, C9, C10, C11, C12, C13_A, C13_B, C13_C, C13_D, C14_A, C14_B, C14_C, C14_D, C15_A, C15_B, C15_C, C15_D, C16_A, C16_B, C16_C, C16_D, C17_A, C17_B, C17_C, C17_D, C18_A, C18_B, C18_C, C18_D</t>
+    <t>C1_A, C1_B, C1_C, C1_D, C4, C5, C6, C7, C8, C9, C10, C11, C12, C13_A, C13_B, C13_C, C13_D, C16_A, C16_B, C16_C, C16_D</t>
   </si>
   <si>
     <t>Samsung Electro-Mechanics</t>
@@ -114,6 +114,21 @@
     <t>C696358</t>
   </si>
   <si>
+    <t>47 nF</t>
+  </si>
+  <si>
+    <t>C14_A, C14_B, C14_C, C14_D, C15_A, C15_B, C15_C, C15_D, C17_A, C17_B, C17_C, C17_D</t>
+  </si>
+  <si>
+    <t>Capacitor 0603, 50 VDC, 47 nF, X7R</t>
+  </si>
+  <si>
+    <t>CL10B473KB8NNNC</t>
+  </si>
+  <si>
+    <t>C1622</t>
+  </si>
+  <si>
     <t>56 pF</t>
   </si>
   <si>
@@ -129,6 +144,27 @@
     <t>C39148</t>
   </si>
   <si>
+    <t>Fuse, 5 A</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>Littlefuse</t>
+  </si>
+  <si>
+    <t>Fuse OMNI BLOK 154</t>
+  </si>
+  <si>
+    <t>0154xxx</t>
+  </si>
+  <si>
+    <t>0154005.DR</t>
+  </si>
+  <si>
+    <t>C206916</t>
+  </si>
+  <si>
     <t>ADA4940-1ARZ-R7</t>
   </si>
   <si>
@@ -210,19 +246,19 @@
     <t>C6285339</t>
   </si>
   <si>
-    <t>REC30K-2415DZ</t>
+    <t>TDK15-24D15W</t>
   </si>
   <si>
     <t>PS2_A, PS2_B, PS2_C, PS2_D</t>
   </si>
   <si>
-    <t>RECOM</t>
-  </si>
-  <si>
-    <t>9-36 V Input, +/- 15 V @1A Output, 30W, isolated DC/DC-converter</t>
-  </si>
-  <si>
-    <t>REC30K</t>
+    <t>TDPOWER</t>
+  </si>
+  <si>
+    <t>Isolated Module DC DC Converter Buck 2 Output ±15V 500mA 9V~36V Input</t>
+  </si>
+  <si>
+    <t>C783530</t>
   </si>
   <si>
     <t>2k</t>
@@ -261,22 +297,22 @@
     <t>C491153</t>
   </si>
   <si>
-    <t>10R</t>
+    <t>8.2R</t>
   </si>
   <si>
     <t>R3_A, R3_B, R3_C, R3_D</t>
   </si>
   <si>
-    <t>KOA Speer</t>
-  </si>
-  <si>
-    <t>SMD 10 ohm 0.5% 0.5W</t>
-  </si>
-  <si>
-    <t>SG73G2BTTD10R0D</t>
-  </si>
-  <si>
-    <t>C5750599</t>
+    <t>UNI-ROYAL(Uniroyal Elec)</t>
+  </si>
+  <si>
+    <t>-55℃~+155℃ 200V 600mW 8.2Ω Thick Film Resistor ±400ppm/℃ ±5% 1206</t>
+  </si>
+  <si>
+    <t>AS0606J082JT5E</t>
+  </si>
+  <si>
+    <t>C966029</t>
   </si>
   <si>
     <t>49R9</t>
@@ -300,6 +336,24 @@
     <t>C114625</t>
   </si>
   <si>
+    <t>0R</t>
+  </si>
+  <si>
+    <t>R8, R9, R10, R11</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL</t>
+  </si>
+  <si>
+    <t>250mW Thick Film Resistors ±800ppm/℃ ±1% 0Ω 1206 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>1206W4F0000T5E</t>
+  </si>
+  <si>
+    <t>C17888</t>
+  </si>
+  <si>
     <t>D-SUB 9, female</t>
   </si>
   <si>
@@ -336,7 +390,7 @@
     <t>M12A-04PMMR-SF7003</t>
   </si>
   <si>
-    <t>X6</t>
+    <t>X6, X7</t>
   </si>
   <si>
     <t>Amphenol</t>
@@ -721,8 +775,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEFA0309-9178-4095-A128-B13B24D8C3CD}">
-  <dimension ref="A1:K16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C618009-16DC-4BBB-A019-057EBB6CFD1C}">
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -774,7 +828,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>11</v>
@@ -836,7 +890,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>24</v>
@@ -867,7 +921,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>29</v>
@@ -876,24 +930,24 @@
         <v>30</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="G5" s="2" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -901,61 +955,61 @@
         <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -963,25 +1017,27 @@
         <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>54</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>55</v>
@@ -989,7 +1045,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>56</v>
@@ -998,48 +1054,50 @@
         <v>57</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="1"/>
       <c r="F9" s="2" t="s">
         <v>59</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="K9" s="1"/>
+        <v>60</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>61</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="E10" s="1"/>
       <c r="F10" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>67</v>
@@ -1047,7 +1105,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>68</v>
@@ -1056,21 +1114,19 @@
         <v>69</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="1"/>
+      <c r="F11" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>72</v>
@@ -1078,7 +1134,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>73</v>
@@ -1096,15 +1152,15 @@
         <v>76</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1112,30 +1168,30 @@
         <v>8</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>82</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="K13" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1143,90 +1199,183 @@
         <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="G14" s="2" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K14" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E16" s="1"/>
       <c r="F16" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>4</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>2</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19" s="1"/>
+      <c r="F19" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M12 Steckverbinder ausgetauscht weil anderer nicht lieferbar. Messwiderstand ausgetauscht weil nicht lieferbar
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_current_measurement_dsub_to_rj45/01/BOM/BOM_JLC-uz_per_current_measurement_dsub_to_rj45.xlsx
+++ b/Project Outputs for uz_per_current_measurement_dsub_to_rj45/01/BOM/BOM_JLC-uz_per_current_measurement_dsub_to_rj45.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_per_current_measurement_dsub_to_rj45_4channel\Project Outputs for uz_per_current_measurement_dsub_to_rj45\01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D69B37AB-5F78-4B31-9E03-C1F2D838A799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{98A76F74-B0C6-440A-A520-9F95CE9507D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{284EEBC3-381F-4E00-B929-186550A49D89}"/>
+    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{3B054C41-8573-4632-BE0F-8806788B6F74}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_current_measurem" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="121">
   <si>
     <t>Quantity</t>
   </si>
@@ -303,16 +303,19 @@
     <t>R3_A, R3_B, R3_C, R3_D</t>
   </si>
   <si>
-    <t>UNI-ROYAL(Uniroyal Elec)</t>
-  </si>
-  <si>
-    <t>-55℃~+155℃ 200V 600mW 8.2Ω Thick Film Resistor ±400ppm/℃ ±5% 1206</t>
-  </si>
-  <si>
-    <t>AS0606J082JT5E</t>
-  </si>
-  <si>
-    <t>C966029</t>
+    <t>YAEGO</t>
+  </si>
+  <si>
+    <t>-55℃~+155℃ 200V 750mW 8.2Ω Thick Film Resistor ±1% ±200ppm/℃ 2010 Chip Resistor</t>
+  </si>
+  <si>
+    <t>RES 2010_5025</t>
+  </si>
+  <si>
+    <t>RC2010FK-078R2L</t>
+  </si>
+  <si>
+    <t>C877647</t>
   </si>
   <si>
     <t>49R9</t>
@@ -387,19 +390,19 @@
     <t>C386758</t>
   </si>
   <si>
-    <t>M12A-04PMMR-SF7003</t>
+    <t>CAZN_M12-P4A-GPL_M12</t>
   </si>
   <si>
     <t>X6, X7</t>
   </si>
   <si>
-    <t>Amphenol</t>
-  </si>
-  <si>
-    <t>M12 Metric Circular Connector, A-Coded, Metal Non-shielded, 4A, 04 pins, Male Connector, Male Contact, Hexagonal, M12*1.0, Screw Thread, PCB 90°, Receptacle, Front Fastened, IP67 Mated</t>
-  </si>
-  <si>
-    <t>C21484133</t>
+    <t>CAZN</t>
+  </si>
+  <si>
+    <t>M12 Metric Circular Connector, A-Coded, Metal Non-shielded, 4A, 04 pins, Male Connector, Male Contact, Hexagonal, M12*1.0, Screw Thread, PCB 90°</t>
+  </si>
+  <si>
+    <t>C19108992</t>
   </si>
 </sst>
 </file>
@@ -775,7 +778,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A53CF1A2-4068-4A82-9909-9DF44FD7AAA9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37FDF8F7-D5B4-4BA2-9BDB-4A40A0DFF5A5}">
   <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1214,15 +1217,15 @@
         <v>88</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1230,30 +1233,30 @@
         <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="F15" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1261,19 +1264,19 @@
         <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="F16" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>77</v>
@@ -1281,10 +1284,10 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1292,30 +1295,30 @@
         <v>4</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="F17" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1323,30 +1326,30 @@
         <v>1</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="F18" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -1354,28 +1357,28 @@
         <v>2</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Output Job erstellt, DFM Tool laufen lassen, kann bestellt werden!
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_current_measurement_dsub_to_rj45/01/BOM/BOM_JLC-uz_per_current_measurement_dsub_to_rj45.xlsx
+++ b/Project Outputs for uz_per_current_measurement_dsub_to_rj45/01/BOM/BOM_JLC-uz_per_current_measurement_dsub_to_rj45.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gauppto\Documents\uz_per_current_measurement_dsub_to_rj45_4channel\Project Outputs for uz_per_current_measurement_dsub_to_rj45\01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98A76F74-B0C6-440A-A520-9F95CE9507D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCA8CAE3-A2D8-4DBB-B2CA-8E0E08493386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{3B054C41-8573-4632-BE0F-8806788B6F74}"/>
+    <workbookView xWindow="20025" yWindow="3090" windowWidth="16245" windowHeight="16320" xr2:uid="{F390C001-437E-4BC7-A247-2652CB78254F}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-uz_per_current_measurem" sheetId="1" r:id="rId1"/>
@@ -778,7 +778,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37FDF8F7-D5B4-4BA2-9BDB-4A40A0DFF5A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D60857BE-3914-4130-BC3E-E8033BB351A4}">
   <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>